<commit_message>
refactor: remove role APIs, add IdP/SAML + Token to API spec
- Remove 8 role management routes from identity.py (project uses groups model, not roles)
- Clean role references from GroupCreate/GroupUpdate/GroupDetailResponse schemas
- Add 9 IdP/SAML management APIs + 1 Token Exchange API to api-spec-v2.xlsx
- Add 2 catch-all path_rules (KB + Rubik) to spec (total: 51 APIs, 34 rules)

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/diagrams/api-spec-v2.xlsx
+++ b/diagrams/api-spec-v2.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="应用接入配置" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'IAM系统接口'!$A$1:$I$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'IAM系统接口'!$A$1:$I$52</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -44,7 +44,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="15">
     <fill>
       <patternFill/>
     </fill>
@@ -106,6 +106,16 @@
         <fgColor rgb="00E4DFEC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D5E8D4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DAE8FC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -133,7 +143,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -172,6 +182,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -540,7 +556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I42"/>
+  <dimension ref="A1:I52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2448,8 +2464,462 @@
       </c>
       <c r="I42" s="5" t="inlineStr"/>
     </row>
+    <row r="43" ht="60" customHeight="1">
+      <c r="A43" s="14" t="inlineStr">
+        <is>
+          <t>IdP管理</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>导入SAML元数据</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/{realm}/idp/saml/import</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>前端</t>
+        </is>
+      </c>
+      <c r="F43" s="5" t="inlineStr">
+        <is>
+          <t>上传SAML元数据XML，解析IdP配置</t>
+        </is>
+      </c>
+      <c r="G43" s="5" t="inlineStr">
+        <is>
+          <t>multipart/form-data file (XML)</t>
+        </is>
+      </c>
+      <c r="H43" s="5" t="inlineStr">
+        <is>
+          <t>SAMLMetadataImportResponse</t>
+        </is>
+      </c>
+      <c r="I43" s="5" t="inlineStr">
+        <is>
+          <t>返回解析出的config字段</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="60" customHeight="1">
+      <c r="A44" s="14" t="inlineStr">
+        <is>
+          <t>IdP管理</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>创建IdP实例</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/{realm}/idp/saml/instances</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>前端</t>
+        </is>
+      </c>
+      <c r="F44" s="5" t="inlineStr">
+        <is>
+          <t>创建SAML IdP实例（每realm仅一个）</t>
+        </is>
+      </c>
+      <c r="G44" s="5" t="inlineStr">
+        <is>
+          <t>{"displayName","enabled","trustEmail","config":{}}</t>
+        </is>
+      </c>
+      <c r="H44" s="5" t="inlineStr">
+        <is>
+          <t>IDPInstanceResponse (201)</t>
+        </is>
+      </c>
+      <c r="I44" s="5" t="inlineStr">
+        <is>
+          <t>alias固定为da-saml-idp</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="60" customHeight="1">
+      <c r="A45" s="14" t="inlineStr">
+        <is>
+          <t>IdP管理</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>修改IdP实例</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/{realm}/idp/saml/instances</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>前端</t>
+        </is>
+      </c>
+      <c r="F45" s="5" t="inlineStr">
+        <is>
+          <t>修改SAML IdP配置</t>
+        </is>
+      </c>
+      <c r="G45" s="5" t="inlineStr">
+        <is>
+          <t>{"displayName","enabled","trustEmail","config":{}}</t>
+        </is>
+      </c>
+      <c r="H45" s="5" t="inlineStr">
+        <is>
+          <t>IDPInstanceResponse</t>
+        </is>
+      </c>
+      <c r="I45" s="5" t="inlineStr"/>
+    </row>
+    <row r="46" ht="60" customHeight="1">
+      <c r="A46" s="14" t="inlineStr">
+        <is>
+          <t>IdP管理</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>IdP实例列表</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/{realm}/idp/saml/instances</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>前端</t>
+        </is>
+      </c>
+      <c r="F46" s="5" t="inlineStr">
+        <is>
+          <t>列出realm下所有IdP实例</t>
+        </is>
+      </c>
+      <c r="G46" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H46" s="5" t="inlineStr">
+        <is>
+          <t>List[IDPInstanceResponse]</t>
+        </is>
+      </c>
+      <c r="I46" s="5" t="inlineStr"/>
+    </row>
+    <row r="47" ht="60" customHeight="1">
+      <c r="A47" s="14" t="inlineStr">
+        <is>
+          <t>IdP管理</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>删除IdP实例</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>DELETE</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/{realm}/idp/saml/instances/{alias}</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>前端</t>
+        </is>
+      </c>
+      <c r="F47" s="5" t="inlineStr">
+        <is>
+          <t>删除指定IdP实例</t>
+        </is>
+      </c>
+      <c r="G47" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H47" s="5" t="inlineStr">
+        <is>
+          <t>204</t>
+        </is>
+      </c>
+      <c r="I47" s="5" t="inlineStr"/>
+    </row>
+    <row r="48" ht="60" customHeight="1">
+      <c r="A48" s="14" t="inlineStr">
+        <is>
+          <t>IdP管理</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>Mapper列表</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/{realm}/idp/saml/instances/{alias}/mappers</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>前端</t>
+        </is>
+      </c>
+      <c r="F48" s="5" t="inlineStr">
+        <is>
+          <t>获取IdP的属性映射列表</t>
+        </is>
+      </c>
+      <c r="G48" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H48" s="5" t="inlineStr">
+        <is>
+          <t>List[IdPMapperResponse]</t>
+        </is>
+      </c>
+      <c r="I48" s="5" t="inlineStr">
+        <is>
+          <t>简化返回</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="60" customHeight="1">
+      <c r="A49" s="14" t="inlineStr">
+        <is>
+          <t>IdP管理</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>创建Mapper</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/{realm}/idp/saml/instances/{alias}/mappers</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>前端</t>
+        </is>
+      </c>
+      <c r="F49" s="5" t="inlineStr">
+        <is>
+          <t>创建属性映射</t>
+        </is>
+      </c>
+      <c r="G49" s="5" t="inlineStr">
+        <is>
+          <t>{"name","attributeKey","attributeValue","friendlyName"}</t>
+        </is>
+      </c>
+      <c r="H49" s="5" t="inlineStr">
+        <is>
+          <t>IdPMapperResponse (201)</t>
+        </is>
+      </c>
+      <c r="I49" s="5" t="inlineStr">
+        <is>
+          <t>固定saml-user-attribute-idp-mapper</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="60" customHeight="1">
+      <c r="A50" s="14" t="inlineStr">
+        <is>
+          <t>IdP管理</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>修改Mapper</t>
+        </is>
+      </c>
+      <c r="C50" s="7" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/{realm}/idp/saml/instances/{alias}/mappers/{mapper_id}</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>前端</t>
+        </is>
+      </c>
+      <c r="F50" s="5" t="inlineStr">
+        <is>
+          <t>修改属性映射</t>
+        </is>
+      </c>
+      <c r="G50" s="5" t="inlineStr">
+        <is>
+          <t>{"name","attributeKey","attributeValue","friendlyName"}</t>
+        </is>
+      </c>
+      <c r="H50" s="5" t="inlineStr">
+        <is>
+          <t>204</t>
+        </is>
+      </c>
+      <c r="I50" s="5" t="inlineStr">
+        <is>
+          <t>部分更新</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="60" customHeight="1">
+      <c r="A51" s="14" t="inlineStr">
+        <is>
+          <t>IdP管理</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>删除Mapper</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>DELETE</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/{realm}/idp/saml/instances/{alias}/mappers/{mapper_id}</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>前端</t>
+        </is>
+      </c>
+      <c r="F51" s="5" t="inlineStr">
+        <is>
+          <t>删除属性映射</t>
+        </is>
+      </c>
+      <c r="G51" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H51" s="5" t="inlineStr">
+        <is>
+          <t>204</t>
+        </is>
+      </c>
+      <c r="I51" s="5" t="inlineStr"/>
+    </row>
+    <row r="52" ht="60" customHeight="1">
+      <c r="A52" s="15" t="inlineStr">
+        <is>
+          <t>Token</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>授权码换Token</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/{realm}/token/exchange</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>前端</t>
+        </is>
+      </c>
+      <c r="F52" s="5" t="inlineStr">
+        <is>
+          <t>OIDC授权码换取access_token</t>
+        </is>
+      </c>
+      <c r="G52" s="5" t="inlineStr">
+        <is>
+          <t>{"code","redirect_uri","client_id","client_secret"}</t>
+        </is>
+      </c>
+      <c r="H52" s="5" t="inlineStr">
+        <is>
+          <t>TokenExchangeResponse</t>
+        </is>
+      </c>
+      <c r="I52" s="5" t="inlineStr">
+        <is>
+          <t>client_secret可选</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I42"/>
+  <autoFilter ref="A1:I52"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2460,7 +2930,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H42"/>
+  <dimension ref="A1:H44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2474,7 +2944,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" s="16" t="inlineStr">
         <is>
           <t>已注册应用</t>
         </is>
@@ -2693,9 +3163,9 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="14" t="inlineStr">
-        <is>
-          <t>路径规则 (path_rules) — 32条</t>
+      <c r="A9" s="16" t="inlineStr">
+        <is>
+          <t>路径规则 (path_rules) — 34条</t>
         </is>
       </c>
     </row>
@@ -3335,37 +3805,37 @@
     </row>
     <row r="34">
       <c r="A34" s="5" t="n">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>rubik</t>
+          <t>knowledgebase</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>/rubik/api/databases/knowledge/special</t>
+          <t>/kb/knowledge_bases/</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>添加特殊知识</t>
+          <t>知识库资源操作（兜底）</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>rubik-admins</t>
+          <t>kb-admins</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>仅rubik-admins可调</t>
+          <t>startswith兜底：捕获所有/{kb_id}/...子路径</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="n">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
@@ -3374,12 +3844,12 @@
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>/rubik/api/config/models/</t>
+          <t>/rubik/api/databases/knowledge/special</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>更新模型预设</t>
+          <t>添加特殊知识</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
@@ -3387,11 +3857,15 @@
           <t>rubik-admins</t>
         </is>
       </c>
-      <c r="F35" s="5" t="inlineStr"/>
+      <c r="F35" s="5" t="inlineStr">
+        <is>
+          <t>仅rubik-admins可调</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
@@ -3400,12 +3874,12 @@
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>/rubik/api/config/database-providers/</t>
+          <t>/rubik/api/config/models/</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>更新数据库提供者</t>
+          <t>更新模型预设</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
@@ -3417,7 +3891,7 @@
     </row>
     <row r="37">
       <c r="A37" s="5" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
@@ -3426,12 +3900,12 @@
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>/rubik/api/config/language</t>
+          <t>/rubik/api/config/database-providers/</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>设置语言</t>
+          <t>更新数据库提供者</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
@@ -3443,7 +3917,7 @@
     </row>
     <row r="38">
       <c r="A38" s="5" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
@@ -3452,12 +3926,12 @@
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>/rubik/api/config/languages</t>
+          <t>/rubik/api/config/language</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>分别设置语言</t>
+          <t>设置语言</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
@@ -3469,7 +3943,7 @@
     </row>
     <row r="39">
       <c r="A39" s="5" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
@@ -3478,12 +3952,12 @@
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>/rubik/api/config/app/</t>
+          <t>/rubik/api/config/languages</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>设置应用配置</t>
+          <t>分别设置语言</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
@@ -3495,7 +3969,7 @@
     </row>
     <row r="40">
       <c r="A40" s="5" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
@@ -3504,12 +3978,12 @@
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>/rubik/api/config/reload</t>
+          <t>/rubik/api/config/app/</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>重载配置</t>
+          <t>设置应用配置</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
@@ -3521,7 +3995,7 @@
     </row>
     <row r="41">
       <c r="A41" s="5" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
@@ -3530,12 +4004,12 @@
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>/rubik/api/config/setup</t>
+          <t>/rubik/api/config/reload</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>初始化配置</t>
+          <t>重载配置</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
@@ -3547,29 +4021,85 @@
     </row>
     <row r="42">
       <c r="A42" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>rubik</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>/rubik/api/config/setup</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>初始化配置</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>rubik-admins</t>
+        </is>
+      </c>
+      <c r="F42" s="5" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="n">
         <v>43</v>
       </c>
-      <c r="B42" s="5" t="inlineStr">
+      <c r="B43" s="5" t="inlineStr">
         <is>
           <t>rubik</t>
         </is>
       </c>
-      <c r="C42" s="5" t="inlineStr">
+      <c r="C43" s="5" t="inlineStr">
         <is>
           <t>/rubik/api/config/llm-providers</t>
         </is>
       </c>
-      <c r="D42" s="5" t="inlineStr">
+      <c r="D43" s="5" t="inlineStr">
         <is>
           <t>LLM提供者管理</t>
         </is>
       </c>
-      <c r="E42" s="5" t="inlineStr">
+      <c r="E43" s="5" t="inlineStr">
         <is>
           <t>rubik-admins</t>
         </is>
       </c>
-      <c r="F42" s="5" t="inlineStr"/>
+      <c r="F43" s="5" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>rubik</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>/rubik/api/databases/</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>数据库资源操作（兜底）</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>rubik-admins</t>
+        </is>
+      </c>
+      <c r="F44" s="5" t="inlineStr">
+        <is>
+          <t>startswith兜底：捕获所有/{db_id}/...子路径</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(idp): add saml-advanced-group-idp-mapper for conditional group assignment
New endpoints under /api/v1/{realm}/idp/saml/instances/{alias}/group-mappers
(GET/POST/PUT/DELETE) wrap Keycloak's saml-advanced-group-idp-mapper to
auto-add SAML users to a Keycloak group when specified attribute conditions
(AND semantics) match, with optional regex matching on values.

Filter existing /mappers list to only return saml-user-attribute-idp-mapper
so the two mapper types stay in their own endpoints.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/diagrams/api-spec-v2.xlsx
+++ b/diagrams/api-spec-v2.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="应用接入配置" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'IAM系统接口'!$A$1:$I$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'IAM系统接口'!$A$1:$I$56</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -556,7 +556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I52"/>
+  <dimension ref="A1:I56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2715,7 +2715,7 @@
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>获取IdP的属性映射列表</t>
+          <t>获取IdP的属性映射列表（saml-user-attribute-idp-mapper）</t>
         </is>
       </c>
       <c r="G48" s="5" t="inlineStr">
@@ -2730,7 +2730,7 @@
       </c>
       <c r="I48" s="5" t="inlineStr">
         <is>
-          <t>简化返回</t>
+          <t>仅返回属性映射类型</t>
         </is>
       </c>
     </row>
@@ -2762,7 +2762,7 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>创建属性映射</t>
+          <t>创建属性映射：SAML属性→Keycloak属性</t>
         </is>
       </c>
       <c r="G49" s="5" t="inlineStr">
@@ -2872,54 +2872,238 @@
       <c r="I51" s="5" t="inlineStr"/>
     </row>
     <row r="52" ht="60" customHeight="1">
-      <c r="A52" s="15" t="inlineStr">
+      <c r="A52" s="14" t="inlineStr">
+        <is>
+          <t>IdP管理</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>GroupMapper列表</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/{realm}/idp/saml/instances/{alias}/group-mappers</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>前端</t>
+        </is>
+      </c>
+      <c r="F52" s="5" t="inlineStr">
+        <is>
+          <t>获取条件化自动加组规则列表（saml-advanced-group-idp-mapper）</t>
+        </is>
+      </c>
+      <c r="G52" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H52" s="5" t="inlineStr">
+        <is>
+          <t>List[IdPGroupMapperResponse]</t>
+        </is>
+      </c>
+      <c r="I52" s="5" t="inlineStr">
+        <is>
+          <t>每条规则：属性条件(AND)+目标组</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="60" customHeight="1">
+      <c r="A53" s="14" t="inlineStr">
+        <is>
+          <t>IdP管理</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>创建GroupMapper</t>
+        </is>
+      </c>
+      <c r="C53" s="6" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/{realm}/idp/saml/instances/{alias}/group-mappers</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>前端</t>
+        </is>
+      </c>
+      <c r="F53" s="5" t="inlineStr">
+        <is>
+          <t>创建条件化自动加组规则：SAML属性命中时自动加入指定组</t>
+        </is>
+      </c>
+      <c r="G53" s="5" t="inlineStr">
+        <is>
+          <t>{"name","conditions":[{"attribute","value"}],"group":"/xxx-admins","regex":false}</t>
+        </is>
+      </c>
+      <c r="H53" s="5" t="inlineStr">
+        <is>
+          <t>IdPGroupMapperResponse (201)</t>
+        </is>
+      </c>
+      <c r="I53" s="5" t="inlineStr">
+        <is>
+          <t>多条件AND，group必须/开头</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="60" customHeight="1">
+      <c r="A54" s="14" t="inlineStr">
+        <is>
+          <t>IdP管理</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>修改GroupMapper</t>
+        </is>
+      </c>
+      <c r="C54" s="7" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/{realm}/idp/saml/instances/{alias}/group-mappers/{mapper_id}</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>前端</t>
+        </is>
+      </c>
+      <c r="F54" s="5" t="inlineStr">
+        <is>
+          <t>修改条件化加组规则</t>
+        </is>
+      </c>
+      <c r="G54" s="5" t="inlineStr">
+        <is>
+          <t>{"name","conditions","group","regex"} 全可选</t>
+        </is>
+      </c>
+      <c r="H54" s="5" t="inlineStr">
+        <is>
+          <t>204</t>
+        </is>
+      </c>
+      <c r="I54" s="5" t="inlineStr">
+        <is>
+          <t>部分更新</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="60" customHeight="1">
+      <c r="A55" s="14" t="inlineStr">
+        <is>
+          <t>IdP管理</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>删除GroupMapper</t>
+        </is>
+      </c>
+      <c r="C55" s="8" t="inlineStr">
+        <is>
+          <t>DELETE</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/{realm}/idp/saml/instances/{alias}/group-mappers/{mapper_id}</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>前端</t>
+        </is>
+      </c>
+      <c r="F55" s="5" t="inlineStr">
+        <is>
+          <t>删除条件化加组规则</t>
+        </is>
+      </c>
+      <c r="G55" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H55" s="5" t="inlineStr">
+        <is>
+          <t>204</t>
+        </is>
+      </c>
+      <c r="I55" s="5" t="inlineStr"/>
+    </row>
+    <row r="56" ht="60" customHeight="1">
+      <c r="A56" s="15" t="inlineStr">
         <is>
           <t>Token</t>
         </is>
       </c>
-      <c r="B52" s="3" t="inlineStr">
+      <c r="B56" s="3" t="inlineStr">
         <is>
           <t>授权码换Token</t>
         </is>
       </c>
-      <c r="C52" s="6" t="inlineStr">
+      <c r="C56" s="6" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="D52" s="5" t="inlineStr">
+      <c r="D56" s="5" t="inlineStr">
         <is>
           <t>/api/v1/{realm}/token/exchange</t>
         </is>
       </c>
-      <c r="E52" s="5" t="inlineStr">
+      <c r="E56" s="5" t="inlineStr">
         <is>
           <t>前端</t>
         </is>
       </c>
-      <c r="F52" s="5" t="inlineStr">
+      <c r="F56" s="5" t="inlineStr">
         <is>
           <t>OIDC授权码换取access_token</t>
         </is>
       </c>
-      <c r="G52" s="5" t="inlineStr">
+      <c r="G56" s="5" t="inlineStr">
         <is>
           <t>{"code","redirect_uri","client_id","client_secret"}</t>
         </is>
       </c>
-      <c r="H52" s="5" t="inlineStr">
+      <c r="H56" s="5" t="inlineStr">
         <is>
           <t>TokenExchangeResponse</t>
         </is>
       </c>
-      <c r="I52" s="5" t="inlineStr">
+      <c r="I56" s="5" t="inlineStr">
         <is>
           <t>client_secret可选</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I52"/>
+  <autoFilter ref="A1:I56"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat(path-rules): support binding multiple groups per rule (OR semantics)
Replace the scalar path_rules.required_group with a path_rule_groups N:M
association table. One rule can now grant access when the caller is in
ANY of the bound groups. CRUD and permission lookups return required_groups[]
aggregated via LEFT JOIN + array_agg. Keep the scalar column as a legacy
NOT NULL fallback to avoid breaking any older readers.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/diagrams/api-spec-v2.xlsx
+++ b/diagrams/api-spec-v2.xlsx
@@ -1823,7 +1823,7 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>所有路径规则（pep-proxy提供）</t>
+          <t>所有路径规则，每条含绑定的 groups 列表</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
@@ -1833,7 +1833,7 @@
       </c>
       <c r="H28" s="5" t="inlineStr">
         <is>
-          <t>List[PathRuleResponse]</t>
+          <t>List[PathRuleResponse] (含required_groups:[])</t>
         </is>
       </c>
       <c r="I28" s="5" t="inlineStr"/>
@@ -1866,12 +1866,12 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>新建路径规则</t>
+          <t>新建路径规则，支持多组 OR 语义</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>{"path_prefix","required_group","description"}</t>
+          <t>{"path_prefix","method?","required_groups":["g1","g2"],"description"}</t>
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr">
@@ -1881,7 +1881,7 @@
       </c>
       <c r="I29" s="5" t="inlineStr">
         <is>
-          <t>通常由init脚本预置</t>
+          <t>required_groups 至少 1 个；method 可为 null</t>
         </is>
       </c>
     </row>
@@ -1913,7 +1913,7 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>单条规则</t>
+          <t>单条规则+绑定的 groups</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
@@ -1956,12 +1956,12 @@
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>修改路径规则</t>
+          <t>修改路径规则；传入 required_groups 时全量替换</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>{"path_prefix","required_group","description"}</t>
+          <t>{"path_prefix?","method?","required_groups?":["g1","g2"],"description?"}</t>
         </is>
       </c>
       <c r="H31" s="5" t="inlineStr">
@@ -1969,7 +1969,11 @@
           <t>PathRuleResponse</t>
         </is>
       </c>
-      <c r="I31" s="5" t="inlineStr"/>
+      <c r="I31" s="5" t="inlineStr">
+        <is>
+          <t>所有字段可选；required_groups 若传则 ≥1</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="60" customHeight="1">
       <c r="A32" s="11" t="inlineStr">
@@ -1999,7 +2003,7 @@
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>删除路径规则</t>
+          <t>删除路径规则（级联删除 path_rule_groups）</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">

</xml_diff>